<commit_message>
new version without table generation
</commit_message>
<xml_diff>
--- a/datagen/params/data_gen.xlsx
+++ b/datagen/params/data_gen.xlsx
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>На листе tables заполните table_name, total_rows, явные target tables, общий write_mode и partition columns по каждому engine.</t>
+          <t>На листе tables заполните table_name, total_rows, явные target tables и общий write_mode.</t>
         </is>
       </c>
     </row>
@@ -1551,24 +1551,24 @@
     <row r="22" ht="44" customHeight="1" s="7">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>hive_partition_columns</t>
+          <t>partition metadata</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Опционально. Список partition columns через запятую для Hive. Обязателен только для OVERWRITE_PARTITIONS.</t>
+          <t>Не задаётся в workbook. Loader читает partition columns из реальной target table только для partition-scoped режимов.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" s="7">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>iceberg_partition_columns</t>
+          <t/>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Опционально. Список partition columns через запятую для Iceberg. Обязателен только для OVERWRITE_PARTITIONS.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Для APPEND и OVERWRITE_TABLE могут быть пустыми. Для OVERWRITE_PARTITIONS обязаны быть заполнены отдельно по каждому engine.</t>
+          <t>OVERWRITE_PARTITIONS и APPEND_DISTINCT_PARTITIONS допустимы только для реально partitioned target tables.</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="24" customWidth="1" style="7" min="1" max="2"/>
@@ -2101,16 +2101,6 @@
           <t>write_mode</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>hive_partition_columns</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>iceberg_partition_columns</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="22" customHeight="1" s="7">
       <c r="A2" s="2" t="inlineStr">
@@ -2136,16 +2126,6 @@
           <t>OVERWRITE_PARTITIONS</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>DATE_PART</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>VALUE_DAY</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="22" customHeight="1" s="7">
       <c r="A3" s="2" t="inlineStr">
@@ -2171,8 +2151,6 @@
           <t>APPEND</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
     </row>
     <row r="6" ht="24" customHeight="1" s="7"/>
   </sheetData>

</xml_diff>

<commit_message>
drop primary key logic and fk -> reference
</commit_message>
<xml_diff>
--- a/datagen/params/data_gen.xlsx
+++ b/datagen/params/data_gen.xlsx
@@ -820,7 +820,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>В sheet таблицы каждая строка должна быть ровно одного типа: generated, foreign key или derived.</t>
+          <t>В sheet таблицы каждая строка должна быть ровно одного типа: generated, reference или derived.</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>generated: заполнены column_name + gen_data_type. output_data_type опционален, остальные специальные поля пустые.</t>
+          <t>generated: заполнены column_name + gen_data_type. output_data_type опционален, reference и derive пустые.</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>foreign key: заполнен только foreign_key. gen_data_type и output_data_type не указываются вручную, constraints допускает только null_ratio.</t>
+          <t>reference: заполнен только reference. gen_data_type и output_data_type не указываются вручную, constraints допускает только null_ratio.</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>derived: заполнены derive + output_data_type. gen_data_type, constraints и foreign_key остаются пустыми.</t>
+          <t>derived: заполнены derive + output_data_type. gen_data_type, constraints и reference остаются пустыми.</t>
         </is>
       </c>
     </row>
@@ -1010,19 +1010,19 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Опционально для generated, обязательно для derived, пусто для foreign key.</t>
+          <t>Опционально для generated, обязательно для derived, пусто для reference.</t>
         </is>
       </c>
     </row>
     <row r="29" s="6">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>is_primary_key</t>
+          <t>removed</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Опционально. TRUE только для generated-колонок. Для PK система сама применяет null_ratio=0 и is_unique=true.</t>
+          <t>Не используется. Уникальность задаётся constraints.is_unique=true.</t>
         </is>
       </c>
     </row>
@@ -1034,19 +1034,19 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Опционально только для generated. Формат key=value; key=value. Для foreign key допустим только null_ratio, для derived поле должно быть пустым.</t>
+          <t>Опционально только для generated. Формат key=value; key=value. Для reference допустим только null_ratio, для derived поле должно быть пустым.</t>
         </is>
       </c>
     </row>
     <row r="31" s="6">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>foreign_key</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Формат: table_name="..."; column_name="..."; relation_type="ONE_TO_MANY|ONE_TO_ONE".</t>
+          <t>Формат: table_name="..."; column_name="..."; cardinality="ONE_TO_MANY|ONE_TO_ONE".</t>
         </is>
       </c>
     </row>
@@ -1215,38 +1215,30 @@
     <row r="48" ht="36" customHeight="1" s="6">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>engine_scope=ICEBERG_ONLY</t>
+          <t>cardinality=ONE_TO_MANY</t>
         </is>
       </c>
       <c r="B48" s="21" t="inlineStr">
         <is>
-          <t>Колонка загружается только в Iceberg. Не возвращайте её в compare SQL или добавьте alias в iceberg_exclude_columns.</t>
+          <t>Reference-колонка может повторять non-null значения родительской колонки.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="36" customHeight="1" s="6">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>relation_type=ONE_TO_MANY</t>
+          <t>cardinality=ONE_TO_ONE</t>
         </is>
       </c>
       <c r="B49" s="21" t="inlineStr">
         <is>
-          <t>FK-колонка может повторять значения родительской колонки.</t>
+          <t>Reference-колонка использует distinct non-null родительские значения без повторов.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="36" customHeight="1" s="6">
-      <c r="A50" s="16" t="inlineStr">
-        <is>
-          <t>relation_type=ONE_TO_ONE</t>
-        </is>
-      </c>
-      <c r="B50" s="21" t="inlineStr">
-        <is>
-          <t>FK-колонка использует родительские значения без повторов; у родителя должно хватить уникальных значений.</t>
-        </is>
-      </c>
+      <c r="A50" s="16" t="n"/>
+      <c r="B50" s="21" t="n"/>
     </row>
     <row r="51" ht="36" customHeight="1" s="6">
       <c r="A51" s="16" t="inlineStr">
@@ -1371,22 +1363,18 @@
     <row r="61" ht="36" customHeight="1" s="6">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>Corner cases</t>
-        </is>
-      </c>
-      <c r="B61" s="18" t="n"/>
+          <t>reference + derive</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>Одновременно запрещены.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="36" customHeight="1" s="6">
-      <c r="A62" s="16" t="inlineStr">
-        <is>
-          <t>foreign_key + derive</t>
-        </is>
-      </c>
-      <c r="B62" s="21" t="inlineStr">
-        <is>
-          <t>Одновременно запрещены.</t>
-        </is>
-      </c>
+      <c r="A62" s="16" t="n"/>
+      <c r="B62" s="21" t="n"/>
     </row>
     <row r="63" ht="36" customHeight="1" s="6">
       <c r="A63" s="16" t="inlineStr">
@@ -1494,7 +1482,7 @@
       </c>
       <c r="J1" s="13" t="inlineStr">
         <is>
-          <t>Foreign Key Example</t>
+          <t>Reference Example</t>
         </is>
       </c>
       <c r="K1" s="13" t="inlineStr">
@@ -1555,7 +1543,7 @@
         <is>
           <t>table_name="company_groups";
 column_name="INN";
-relation_type="ONE_TO_MANY|ONE_TO_ONE"</t>
+cardinality="ONE_TO_MANY|ONE_TO_ONE"</t>
         </is>
       </c>
       <c r="K2" s="13" t="inlineStr">
@@ -1734,7 +1722,7 @@
       </c>
       <c r="Q6" s="21" t="inlineStr">
         <is>
-          <t>Итоговый тип. Обязателен для derived, пустой для foreign_key.</t>
+          <t>Итоговый тип. Обязателен для derived, пустой для reference.</t>
         </is>
       </c>
     </row>
@@ -1766,12 +1754,12 @@
     <row r="8" ht="44" customHeight="1" s="6">
       <c r="P8" s="16" t="inlineStr">
         <is>
-          <t>foreign_key</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="Q8" s="21" t="inlineStr">
         <is>
-          <t>table_name="..."; column_name="..."; relation_type="ONE_TO_MANY|ONE_TO_ONE".</t>
+          <t>table_name="..."; column_name="..."; cardinality="ONE_TO_MANY|ONE_TO_ONE".</t>
         </is>
       </c>
     </row>
@@ -2039,11 +2027,7 @@
           <t>output_data_type</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
-        <is>
-          <t>is_primary_key</t>
-        </is>
-      </c>
+      <c r="D1" s="10" t="n"/>
       <c r="E1" s="10" t="inlineStr">
         <is>
           <t>constraints</t>
@@ -2051,7 +2035,7 @@
       </c>
       <c r="F1" s="10" t="inlineStr">
         <is>
-          <t>foreign_key</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="G1" s="10" t="inlineStr">
@@ -2071,7 +2055,7 @@
       </c>
       <c r="J1" s="11" t="inlineStr">
         <is>
-          <t>Пример заполнения foreign_key</t>
+          <t>Пример заполнения reference</t>
         </is>
       </c>
       <c r="K1" s="12" t="inlineStr">
@@ -2092,12 +2076,10 @@
         </is>
       </c>
       <c r="C2" s="8" t="n"/>
-      <c r="D2" s="8" t="b">
-        <v>1</v>
-      </c>
+      <c r="D2" s="8" t="n"/>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>digits_count=10</t>
+          <t>digits_count=10; is_unique=true</t>
         </is>
       </c>
       <c r="F2" s="8" t="n"/>
@@ -2108,7 +2090,7 @@
       </c>
       <c r="H2" s="8" t="n"/>
       <c r="I2" s="7">
-        <f>IF($F2&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H2&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B2,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F2&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H2&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B2,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J2" s="7">
@@ -2146,7 +2128,7 @@
       </c>
       <c r="H3" s="8" t="n"/>
       <c r="I3" s="7">
-        <f>IF($F3&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H3&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B3,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F3&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H3&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B3,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J3" s="7">
@@ -2184,7 +2166,7 @@
       </c>
       <c r="H4" s="8" t="n"/>
       <c r="I4" s="7">
-        <f>IF($F4&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H4&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B4,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F4&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H4&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B4,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J4" s="7">
@@ -2222,7 +2204,7 @@
       </c>
       <c r="H5" s="8" t="n"/>
       <c r="I5" s="7">
-        <f>IF($F5&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H5&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B5,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F5&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H5&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B5,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J5" s="7">
@@ -2260,7 +2242,7 @@
         </is>
       </c>
       <c r="I6" s="7">
-        <f>IF($F6&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H6&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B6,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F6&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H6&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B6,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J6" s="7">
@@ -2326,11 +2308,7 @@
           <t>output_data_type</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
-        <is>
-          <t>is_primary_key</t>
-        </is>
-      </c>
+      <c r="D1" s="10" t="n"/>
       <c r="E1" s="10" t="inlineStr">
         <is>
           <t>constraints</t>
@@ -2338,7 +2316,7 @@
       </c>
       <c r="F1" s="10" t="inlineStr">
         <is>
-          <t>foreign_key</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="G1" s="10" t="inlineStr">
@@ -2358,7 +2336,7 @@
       </c>
       <c r="J1" s="11" t="inlineStr">
         <is>
-          <t>Пример заполнения foreign_key</t>
+          <t>Пример заполнения reference</t>
         </is>
       </c>
       <c r="K1" s="12" t="inlineStr">
@@ -2393,7 +2371,7 @@
       </c>
       <c r="H2" s="8" t="n"/>
       <c r="I2" s="7">
-        <f>IF($F2&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H2&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B2,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F2&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H2&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B2,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J2" s="7">
@@ -2417,7 +2395,7 @@
       <c r="E3" s="8" t="n"/>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>table_name="company_groups"; column_name="INN"; relation_type="ONE_TO_MANY"</t>
+          <t>table_name="company_groups"; column_name="INN"; cardinality="ONE_TO_MANY"</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -2427,7 +2405,7 @@
       </c>
       <c r="H3" s="8" t="n"/>
       <c r="I3" s="7">
-        <f>IF($F3&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H3&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B3,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F3&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H3&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B3,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J3" s="7">
@@ -2465,7 +2443,7 @@
       </c>
       <c r="H4" s="8" t="n"/>
       <c r="I4" s="7">
-        <f>IF($F4&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H4&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B4,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F4&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H4&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B4,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J4" s="7">
@@ -2503,7 +2481,7 @@
       </c>
       <c r="H5" s="8" t="n"/>
       <c r="I5" s="7">
-        <f>IF($F5&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H5&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B5,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F5&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H5&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B5,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J5" s="7">
@@ -2541,7 +2519,7 @@
       </c>
       <c r="H6" s="8" t="n"/>
       <c r="I6" s="7">
-        <f>IF($F6&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H6&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B6,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F6&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H6&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B6,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J6" s="7">
@@ -2579,7 +2557,7 @@
       </c>
       <c r="H7" s="8" t="n"/>
       <c r="I7" s="7">
-        <f>IF($F7&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H7&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B7,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F7&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H7&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B7,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J7" s="7">
@@ -2617,7 +2595,7 @@
       </c>
       <c r="H8" s="8" t="n"/>
       <c r="I8" s="7">
-        <f>IF($F8&lt;&gt;"","Для foreign_key допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H8&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/foreign_key оставьте пустыми.",IFERROR(VLOOKUP($B8,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
+        <f>IF($F8&lt;&gt;"","Для reference допустим только null_ratio=0..1. gen_data_type и output_data_type выводятся из parent column.",IF($H8&lt;&gt;"","Для derive укажите output_data_type и engine_scope; доступные rule: YYYYMMDD|YYYY|MM; gen_data_type/constraints/reference оставьте пустыми.",IFERROR(VLOOKUP($B8,'Constant List'!$A$2:$B$7,2,FALSE),"Тип генерации не заполнен")))</f>
         <v/>
       </c>
       <c r="J8" s="7">

</xml_diff>